<commit_message>
Added & update the code for the calling feature
</commit_message>
<xml_diff>
--- a/src/test/resources/TestDataFile.xlsx
+++ b/src/test/resources/TestDataFile.xlsx
@@ -4,12 +4,13 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12180" activeTab="1"/>
+    <workbookView windowWidth="28800" windowHeight="12180" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="VerifyLogin" sheetId="1" r:id="rId1"/>
     <sheet name="VerifyLoginWithInvalidData" sheetId="3" r:id="rId2"/>
     <sheet name="verifySignUp" sheetId="2" r:id="rId3"/>
+    <sheet name="VerifyEngageTab" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="23">
   <si>
     <t>loginUsername</t>
   </si>
@@ -37,55 +38,67 @@
     <t>loginPassword</t>
   </si>
   <si>
+    <t xml:space="preserve"> moonlivesub40+877@gmail.com</t>
+  </si>
+  <si>
+    <t>test@1234567</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>moonlivesub</t>
+  </si>
+  <si>
+    <t>moonlivesub40+71@@gmail.com</t>
+  </si>
+  <si>
+    <t>moonlivesub40+71gmail.com</t>
+  </si>
+  <si>
+    <t>moonlivesub40+71@gmail</t>
+  </si>
+  <si>
+    <t>moonlivesub40+73@gmail.com</t>
+  </si>
+  <si>
+    <t>emailID</t>
+  </si>
+  <si>
+    <t>FirstName</t>
+  </si>
+  <si>
+    <t>LastName</t>
+  </si>
+  <si>
+    <t>Password</t>
+  </si>
+  <si>
+    <t>ConfirmPassword</t>
+  </si>
+  <si>
+    <t>{faker.email}</t>
+  </si>
+  <si>
+    <t>{faker.firstName}</t>
+  </si>
+  <si>
+    <t>{faker.lastName}</t>
+  </si>
+  <si>
+    <t>{faker.Password}</t>
+  </si>
+  <si>
+    <t>receiverUsername</t>
+  </si>
+  <si>
+    <t>receiverPassword</t>
+  </si>
+  <si>
     <t>qa1+20022026@moontechnolabs.com</t>
   </si>
   <si>
     <t>Test@12345</t>
-  </si>
-  <si>
-    <t>Email</t>
-  </si>
-  <si>
-    <t>moonlivesub</t>
-  </si>
-  <si>
-    <t>moonlivesub40+71@@gmail.com</t>
-  </si>
-  <si>
-    <t>moonlivesub40+71gmail.com</t>
-  </si>
-  <si>
-    <t>moonlivesub40+71@gmail</t>
-  </si>
-  <si>
-    <t>moonlivesub40+73@gmail.com</t>
-  </si>
-  <si>
-    <t>emailID</t>
-  </si>
-  <si>
-    <t>FirstName</t>
-  </si>
-  <si>
-    <t>LastName</t>
-  </si>
-  <si>
-    <t>Password</t>
-  </si>
-  <si>
-    <t>ConfirmPassword</t>
-  </si>
-  <si>
-    <t>{faker.email}</t>
-  </si>
-  <si>
-    <t>{faker.firstName}</t>
-  </si>
-  <si>
-    <t>{faker.lastName}</t>
-  </si>
-  <si>
-    <t>{faker.Password}</t>
   </si>
 </sst>
 </file>
@@ -93,10 +106,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
   <numFmts count="4">
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="179" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
   </numFmts>
   <fonts count="20">
     <font>
@@ -559,16 +572,16 @@
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -701,7 +714,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -715,6 +728,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1275,7 +1291,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" display="Test@12345"/>
+    <hyperlink ref="B2" r:id="rId1" display="test@1234567" tooltip="mailto:test@1234567"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
@@ -1375,4 +1391,54 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="3"/>
+  <cols>
+    <col min="1" max="1" width="32.7142857142857" customWidth="1"/>
+    <col min="2" max="2" width="26.2857142857143" customWidth="1"/>
+    <col min="3" max="3" width="36.1428571428571" customWidth="1"/>
+    <col min="4" max="4" width="22.5714285714286" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" s="1" customFormat="1" spans="1:4">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" s="1" customFormat="1" spans="1:4">
+      <c r="A2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" display="test@1234567" tooltip="mailto:test@1234567"/>
+    <hyperlink ref="D2" r:id="rId2" display="Test@12345"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Added & update the code
</commit_message>
<xml_diff>
--- a/src/test/resources/TestDataFile.xlsx
+++ b/src/test/resources/TestDataFile.xlsx
@@ -4,13 +4,15 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12180" activeTab="3"/>
+    <workbookView windowWidth="28800" windowHeight="12180" firstSheet="1" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="VerifyLogin" sheetId="1" r:id="rId1"/>
     <sheet name="VerifyLoginWithInvalidData" sheetId="3" r:id="rId2"/>
     <sheet name="verifySignUp" sheetId="2" r:id="rId3"/>
     <sheet name="VerifyEngageTab" sheetId="4" r:id="rId4"/>
+    <sheet name="VerifyEngageChat" sheetId="5" r:id="rId5"/>
+    <sheet name="VerifySettingPage" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="26">
   <si>
     <t>loginUsername</t>
   </si>
@@ -99,6 +101,15 @@
   </si>
   <si>
     <t>Test@12345</t>
+  </si>
+  <si>
+    <t>dummyMessage</t>
+  </si>
+  <si>
+    <t>moonlivesub40+877@gmail.com</t>
+  </si>
+  <si>
+    <t>{faker.dummyMessage}</t>
   </si>
 </sst>
 </file>
@@ -718,9 +729,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -728,6 +736,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6" applyAlignment="1">
@@ -1274,18 +1285,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>3</v>
       </c>
     </row>
@@ -1356,34 +1367,34 @@
     <col min="5" max="5" width="18.1428571428571" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" spans="1:5">
-      <c r="A1" s="1" t="s">
+    <row r="1" s="4" customFormat="1" spans="1:5">
+      <c r="A1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="2" s="1" customFormat="1" spans="1:4">
-      <c r="A2" s="1" t="s">
+    <row r="2" s="4" customFormat="1" spans="1:4">
+      <c r="A2" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="4" t="s">
         <v>18</v>
       </c>
     </row>
@@ -1405,28 +1416,28 @@
     <col min="4" max="4" width="22.5714285714286" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" spans="1:4">
-      <c r="A1" s="2" t="s">
+    <row r="1" s="4" customFormat="1" spans="1:4">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="4" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="2" s="1" customFormat="1" spans="1:4">
-      <c r="A2" s="3" t="s">
+    <row r="2" s="4" customFormat="1" spans="1:4">
+      <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="4" t="s">
         <v>21</v>
       </c>
       <c r="D2" s="5" t="s">
@@ -1441,4 +1452,81 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="2"/>
+  <cols>
+    <col min="1" max="1" width="31.8571428571429" customWidth="1"/>
+    <col min="2" max="2" width="19.5714285714286" customWidth="1"/>
+    <col min="3" max="3" width="39.8571428571429" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" display="test@1234567" tooltip="mailto:test@1234567"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="1"/>
+  <cols>
+    <col min="1" max="1" width="35.1428571428571" customWidth="1"/>
+    <col min="2" max="2" width="27.4285714285714" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" display="test@1234567" tooltip="mailto:test@1234567"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
 </file>
</xml_diff>